<commit_message>
test: add pytest suite for protobuf parsers and single-source version
</commit_message>
<xml_diff>
--- a/sample/多帖汇总示例.xlsx
+++ b/sample/多帖汇总示例.xlsx
@@ -845,7 +845,7 @@
       </c>
       <c r="B10" s="25" t="inlineStr">
         <is>
-          <t>2026-10-18 06:04:41</t>
+          <t>2026-10-18 06:37:59</t>
         </is>
       </c>
     </row>
@@ -2738,7 +2738,7 @@
       </c>
       <c r="B10" s="25" t="inlineStr">
         <is>
-          <t>2026-10-18 06:04:41</t>
+          <t>2026-10-18 06:37:59</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
style: apply ruff format
</commit_message>
<xml_diff>
--- a/sample/多帖汇总示例.xlsx
+++ b/sample/多帖汇总示例.xlsx
@@ -845,7 +845,7 @@
       </c>
       <c r="B10" s="25" t="inlineStr">
         <is>
-          <t>2026-10-18 06:37:59</t>
+          <t>2026-10-18 14:41:01</t>
         </is>
       </c>
     </row>
@@ -2738,7 +2738,7 @@
       </c>
       <c r="B10" s="25" t="inlineStr">
         <is>
-          <t>2026-10-18 06:37:59</t>
+          <t>2026-10-18 14:41:01</t>
         </is>
       </c>
     </row>

</xml_diff>